<commit_message>
chore: sync from internal mirror (96a02f4)
</commit_message>
<xml_diff>
--- a/packages/calculators/src/modules/test/15.2-purchased-feed.xlsx
+++ b/packages/calculators/src/modules/test/15.2-purchased-feed.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11018"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mackcheesman/Desktop/Work/EAP/Code/emissions-calculators/packages/calculators/src/modules/test/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eddiesholl/Code/aginnovationaustralia/emissions-calculators-internal/packages/calculators/src/modules/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5D84356-6055-D449-AE38-2FED63AD1F8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7E8D6A1-EFDA-FF41-BDD1-2770A70F6A6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1820" yWindow="1500" windowWidth="25020" windowHeight="13000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -719,18 +719,18 @@
       </c>
       <c r="D11">
         <f>I11</f>
-        <v>0.38600000000000001</v>
+        <v>0.41</v>
       </c>
       <c r="E11">
         <f>C11*D11</f>
-        <v>38.6</v>
+        <v>41</v>
       </c>
       <c r="G11" s="5" t="s">
         <v>14</v>
       </c>
       <c r="H11" s="5"/>
       <c r="I11" s="5">
-        <v>0.38600000000000001</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.2">
@@ -742,18 +742,18 @@
       </c>
       <c r="D12">
         <f t="shared" ref="D12:D75" si="0">I12</f>
-        <v>1.9</v>
+        <v>0.41</v>
       </c>
       <c r="E12">
         <f t="shared" ref="E12:E75" si="1">C12*D12</f>
-        <v>380</v>
+        <v>82</v>
       </c>
       <c r="G12" s="5" t="s">
         <v>15</v>
       </c>
       <c r="H12" s="5"/>
       <c r="I12" s="5">
-        <v>1.9</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>